<commit_message>
adding search feature on RM AKTIF,INAKTIF and PASIEN DATA
</commit_message>
<xml_diff>
--- a/proses/Pasien.xlsx
+++ b/proses/Pasien.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
   <si>
     <t>NO</t>
   </si>
@@ -44,64 +44,46 @@
     <t>ALAMAT</t>
   </si>
   <si>
-    <t>Arif W</t>
-  </si>
-  <si>
-    <t>dipo</t>
+    <t>ALIP DUGONG</t>
+  </si>
+  <si>
+    <t>rujuk sanyoto</t>
   </si>
   <si>
     <t>Laki Laki</t>
   </si>
   <si>
-    <t>Karyawan</t>
-  </si>
-  <si>
-    <t>2006-02-23</t>
+    <t>CAPLIN</t>
+  </si>
+  <si>
+    <t>2022-02-09</t>
+  </si>
+  <si>
+    <t>RADEU AGAMA</t>
+  </si>
+  <si>
+    <t>CABEAN SISIH DUWUR</t>
+  </si>
+  <si>
+    <t>Jumirah</t>
+  </si>
+  <si>
+    <t>Slamet</t>
+  </si>
+  <si>
+    <t>Perempuan</t>
+  </si>
+  <si>
+    <t>TKW</t>
+  </si>
+  <si>
+    <t>2005-02-28</t>
   </si>
   <si>
     <t>Islam</t>
   </si>
   <si>
-    <t>Ngelo Tegalwaton</t>
-  </si>
-  <si>
-    <t>Fajar</t>
-  </si>
-  <si>
-    <t>rujuk sanyoto</t>
-  </si>
-  <si>
-    <t>2001-02-28</t>
-  </si>
-  <si>
-    <t>MAGELANG</t>
-  </si>
-  <si>
-    <t>Painah Juminem</t>
-  </si>
-  <si>
-    <t>Perempuan</t>
-  </si>
-  <si>
-    <t>Ibu Rumah Tangga</t>
-  </si>
-  <si>
-    <t>2012-07-01</t>
-  </si>
-  <si>
-    <t>TEGALGEDE</t>
-  </si>
-  <si>
-    <t>Emiyati</t>
-  </si>
-  <si>
-    <t>basirun</t>
-  </si>
-  <si>
-    <t>1997-07-25</t>
-  </si>
-  <si>
-    <t>Ngelo</t>
+    <t>Sunggingan</t>
   </si>
 </sst>
 </file>
@@ -441,7 +423,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -478,7 +460,7 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>3323323</v>
+        <v>783687368</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
@@ -507,7 +489,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>8890908</v>
+        <v>328973298237</v>
       </c>
       <c r="C3" t="s">
         <v>16</v>
@@ -516,77 +498,19 @@
         <v>17</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>33422345</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F4" t="s">
         <v>22</v>
-      </c>
-      <c r="G4" t="s">
-        <v>23</v>
-      </c>
-      <c r="H4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5">
-        <v>9909989989</v>
-      </c>
-      <c r="C5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G5" t="s">
-        <v>27</v>
-      </c>
-      <c r="H5" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" t="s">
-        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding pdf open, adding edit all pasien
</commit_message>
<xml_diff>
--- a/proses/Pasien.xlsx
+++ b/proses/Pasien.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="28">
   <si>
     <t>NO</t>
   </si>
@@ -84,6 +84,21 @@
   </si>
   <si>
     <t>Sunggingan</t>
+  </si>
+  <si>
+    <t>Surya dewa</t>
+  </si>
+  <si>
+    <t>Mbah Onggo</t>
+  </si>
+  <si>
+    <t>Buruh</t>
+  </si>
+  <si>
+    <t>2001-07-28</t>
+  </si>
+  <si>
+    <t>Dukuh Kranggan</t>
   </si>
 </sst>
 </file>
@@ -423,7 +438,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -511,6 +526,35 @@
       </c>
       <c r="I3" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>767866576576</v>
+      </c>
+      <c r="C4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="I4" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>